<commit_message>
KPI actualizado 2026-07-06 22:01 UTC
</commit_message>
<xml_diff>
--- a/data/50001558 - GESVIAL OT4342-4344.xlsx
+++ b/data/50001558 - GESVIAL OT4342-4344.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1472" uniqueCount="376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1439" uniqueCount="365">
   <si>
     <t>50001558 -  GESVIAL</t>
   </si>
@@ -719,7 +719,7 @@
     <t>1215174260169824</t>
   </si>
   <si>
-    <t>OT 4344 - MANGA DE VENTILACION Ø1600MM,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,OT 4344 - MANGA DE VENTILACION Ø1600MM,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,Propuesta Mecanizado,Propuesta Fabricación externa ,propuesta Corte Laser,Propuesta Corte plasma ,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A</t>
+    <t>OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,Propuesta Mecanizado,Propuesta Fabricación externa ,propuesta Corte Laser,Propuesta Corte plasma ,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A</t>
   </si>
   <si>
     <t>1215174141207989</t>
@@ -776,7 +776,7 @@
     <t>Recepcion materiales corte laser,Recepcion Materiales corte plasma</t>
   </si>
   <si>
-    <t>OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,OT 4344 - MANGA DE VENTILACION Ø1600MM x 50,Bodega:</t>
+    <t>OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,Bodega:</t>
   </si>
   <si>
     <t>1215174260282365</t>
@@ -794,9 +794,6 @@
     <t>Control de calidad Corte plasma</t>
   </si>
   <si>
-    <t>OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,OT 4344 - MANGA DE VENTILACION Ø1600MM x 50</t>
-  </si>
-  <si>
     <t>1215174141283554</t>
   </si>
   <si>
@@ -842,15 +839,6 @@
     <t>Preparación Materiales,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A</t>
   </si>
   <si>
-    <t>1215174166752264</t>
-  </si>
-  <si>
-    <t>OT 4344 - MANGA DE VENTILACION Ø1600MM x 50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Control de calidad Corte plasma,Control de calidad Mecanizado,control de calidad corte laser </t>
-  </si>
-  <si>
     <t>1215174266589473</t>
   </si>
   <si>
@@ -866,15 +854,6 @@
     <t>Armado,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A</t>
   </si>
   <si>
-    <t>1215174166783266</t>
-  </si>
-  <si>
-    <t>OT 4344 - MANGA DE VENTILACION Ø1600MM x 50,check planos</t>
-  </si>
-  <si>
-    <t>Armado,OT 4344 - MANGA DE VENTILACION Ø1600MM</t>
-  </si>
-  <si>
     <t>1215174382789626</t>
   </si>
   <si>
@@ -887,15 +866,6 @@
     <t>Control de calidad Armado,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A</t>
   </si>
   <si>
-    <t>1215174141334795</t>
-  </si>
-  <si>
-    <t>OT 4344 - MANGA DE VENTILACION Ø1600MM,check planos</t>
-  </si>
-  <si>
-    <t>Control de calidad Armado,OT 4344 - MANGA DE VENTILACION Ø1600MM</t>
-  </si>
-  <si>
     <t>1215174266619637</t>
   </si>
   <si>
@@ -906,9 +876,6 @@
   </si>
   <si>
     <t>Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,Bodega:</t>
   </si>
   <si>
     <t>1215174266650610</t>
@@ -1702,7 +1669,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U123"/>
+  <dimension ref="A1:U120"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -5230,7 +5197,7 @@
         <v>46196.87995266204</v>
       </c>
       <c r="D61" s="9">
-        <v>46196.879968090274</v>
+        <v>46209.908330949074</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>97</v>
@@ -5574,7 +5541,7 @@
       </c>
       <c r="C67" s="10"/>
       <c r="D67" s="9">
-        <v>46174.847163576385</v>
+        <v>46209.90823064814</v>
       </c>
       <c r="E67" s="10" t="s">
         <v>239</v>
@@ -5700,7 +5667,7 @@
       </c>
       <c r="C69" s="10"/>
       <c r="D69" s="9">
-        <v>46174.84716077546</v>
+        <v>46209.90823061342</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>246</v>
@@ -5736,7 +5703,7 @@
         <v>243</v>
       </c>
       <c r="P69" s="10" t="s">
-        <v>247</v>
+        <v>206</v>
       </c>
       <c r="Q69" s="9">
         <v>46260</v>
@@ -5756,7 +5723,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B70" s="5">
         <v>46169.669448368055</v>
@@ -5766,7 +5733,7 @@
         <v>46199.57084185185</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
@@ -5799,7 +5766,7 @@
         <v>194</v>
       </c>
       <c r="P70" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="Q70" s="5">
         <v>46258</v>
@@ -5819,17 +5786,17 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B71" s="9">
         <v>46169.66945298611</v>
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="9">
-        <v>46174.847156944445</v>
+        <v>46209.90823069445</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>26</v>
@@ -5859,10 +5826,10 @@
         <v>231</v>
       </c>
       <c r="O71" s="10" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="P71" s="10" t="s">
-        <v>247</v>
+        <v>206</v>
       </c>
       <c r="Q71" s="9">
         <v>46260</v>
@@ -5882,17 +5849,17 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B72" s="5">
         <v>46169.66945778935</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46170.62754262731</v>
+        <v>46209.909264270835</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>25</v>
@@ -5916,7 +5883,7 @@
         <v>26</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="P72" s="6" t="s">
         <v>26</v>
@@ -5929,26 +5896,28 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B73" s="9">
         <v>46169.66946104167</v>
       </c>
-      <c r="C73" s="10"/>
+      <c r="C73" s="9">
+        <v>46209.90925715277</v>
+      </c>
       <c r="D73" s="9">
-        <v>46174.84730037037</v>
+        <v>46209.90937729167</v>
       </c>
       <c r="E73" s="10" t="s">
+        <v>255</v>
+      </c>
+      <c r="F73" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G73" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="F73" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G73" s="10" t="s">
+      <c r="H73" s="10" t="s">
         <v>257</v>
-      </c>
-      <c r="H73" s="10" t="s">
-        <v>258</v>
       </c>
       <c r="I73" s="9">
         <v>46262</v>
@@ -5966,13 +5935,13 @@
         <v>26</v>
       </c>
       <c r="N73" s="10" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O73" s="10" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="P73" s="10" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="Q73" s="9">
         <v>46262</v>
@@ -5984,22 +5953,24 @@
         <v>33</v>
       </c>
       <c r="T73" s="10">
-        <v>0</v>
-      </c>
-      <c r="U73" s="11" t="s">
-        <v>60</v>
+        <v>1</v>
+      </c>
+      <c r="U73" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B74" s="5">
         <v>46169.669467280095</v>
       </c>
-      <c r="C74" s="6"/>
+      <c r="C74" s="5">
+        <v>46209.909371331014</v>
+      </c>
       <c r="D74" s="5">
-        <v>46174.84726460648</v>
+        <v>46209.90937271991</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>206</v>
@@ -6008,10 +5979,10 @@
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="H74" s="6" t="s">
         <v>257</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>258</v>
       </c>
       <c r="I74" s="5">
         <v>46262</v>
@@ -6029,13 +6000,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="O74" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="P74" s="6" t="s">
         <v>261</v>
-      </c>
-      <c r="P74" s="6" t="s">
-        <v>262</v>
       </c>
       <c r="Q74" s="6"/>
       <c r="R74" s="6"/>
@@ -6045,32 +6016,32 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="8" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B75" s="9">
-        <v>46169.66947349537</v>
+        <v>46169.66950289352</v>
       </c>
       <c r="C75" s="10"/>
       <c r="D75" s="9">
-        <v>46174.84726170139</v>
+        <v>46209.90954123843</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G75" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="H75" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="H75" s="10" t="s">
-        <v>258</v>
-      </c>
       <c r="I75" s="9">
-        <v>46262</v>
+        <v>46273</v>
       </c>
       <c r="J75" s="9">
-        <v>46272</v>
+        <v>46293</v>
       </c>
       <c r="K75" s="10" t="s">
         <v>26</v>
@@ -6082,42 +6053,52 @@
         <v>26</v>
       </c>
       <c r="N75" s="10" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="O75" s="10" t="s">
-        <v>265</v>
+        <v>206</v>
       </c>
       <c r="P75" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="Q75" s="10"/>
-      <c r="R75" s="10"/>
-      <c r="S75" s="10"/>
-      <c r="T75" s="10"/>
-      <c r="U75" s="10"/>
+        <v>252</v>
+      </c>
+      <c r="Q75" s="9">
+        <v>46273</v>
+      </c>
+      <c r="R75" s="9">
+        <v>46293</v>
+      </c>
+      <c r="S75" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T75" s="10">
+        <v>0.1</v>
+      </c>
+      <c r="U75" s="12" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B76" s="5">
-        <v>46169.66950289352</v>
+        <v>46169.66950758102</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46174.847443506944</v>
+        <v>46209.90937868056</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>267</v>
+        <v>206</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="H76" s="6" t="s">
         <v>257</v>
-      </c>
-      <c r="H76" s="6" t="s">
-        <v>258</v>
       </c>
       <c r="I76" s="5">
         <v>46273</v>
@@ -6135,111 +6116,109 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>253</v>
+        <v>263</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>204</v>
+        <v>265</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>253</v>
-      </c>
-      <c r="Q76" s="5">
-        <v>46273</v>
-      </c>
-      <c r="R76" s="5">
-        <v>46293</v>
-      </c>
-      <c r="S76" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T76" s="6">
-        <v>0</v>
-      </c>
-      <c r="U76" s="11" t="s">
-        <v>60</v>
-      </c>
+        <v>266</v>
+      </c>
+      <c r="Q76" s="6"/>
+      <c r="R76" s="6"/>
+      <c r="S76" s="6"/>
+      <c r="T76" s="6"/>
+      <c r="U76" s="6"/>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B77" s="9">
-        <v>46169.66950758102</v>
+        <v>46169.66953380787</v>
       </c>
       <c r="C77" s="10"/>
       <c r="D77" s="9">
-        <v>46196.87995929398</v>
+        <v>46209.908330833336</v>
       </c>
       <c r="E77" s="10" t="s">
+        <v>268</v>
+      </c>
+      <c r="F77" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G77" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="H77" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="I77" s="9">
+        <v>46294</v>
+      </c>
+      <c r="J77" s="9">
+        <v>46294</v>
+      </c>
+      <c r="K77" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="L77" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="M77" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="N77" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="O77" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="F77" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G77" s="10" t="s">
-        <v>257</v>
-      </c>
-      <c r="H77" s="10" t="s">
-        <v>258</v>
-      </c>
-      <c r="I77" s="9">
-        <v>46273</v>
-      </c>
-      <c r="J77" s="9">
-        <v>46293</v>
-      </c>
-      <c r="K77" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="L77" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="M77" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="N77" s="10" t="s">
-        <v>267</v>
-      </c>
-      <c r="O77" s="10" t="s">
-        <v>269</v>
-      </c>
       <c r="P77" s="10" t="s">
-        <v>270</v>
-      </c>
-      <c r="Q77" s="10"/>
-      <c r="R77" s="10"/>
-      <c r="S77" s="10"/>
-      <c r="T77" s="10"/>
-      <c r="U77" s="10"/>
+        <v>252</v>
+      </c>
+      <c r="Q77" s="9">
+        <v>46294</v>
+      </c>
+      <c r="R77" s="9">
+        <v>46294</v>
+      </c>
+      <c r="S77" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T77" s="10">
+        <v>0</v>
+      </c>
+      <c r="U77" s="11" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B78" s="5">
-        <v>46169.66951364583</v>
+        <v>46169.66953854167</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46196.87995984954</v>
+        <v>46197.84256122685</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>257</v>
+        <v>186</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="I78" s="5">
-        <v>46273</v>
-      </c>
+        <v>187</v>
+      </c>
+      <c r="I78" s="6"/>
       <c r="J78" s="5">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="K78" s="6" t="s">
         <v>26</v>
@@ -6251,13 +6230,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="Q78" s="6"/>
       <c r="R78" s="6"/>
@@ -6267,33 +6246,27 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="B79" s="9">
-        <v>46169.66953380787</v>
+        <v>46169.66960108797</v>
       </c>
       <c r="C79" s="10"/>
       <c r="D79" s="9">
-        <v>46197.84261425926</v>
+        <v>46209.85402508102</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>275</v>
+        <v>231</v>
       </c>
       <c r="F79" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G79" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="H79" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="I79" s="9">
-        <v>46294</v>
-      </c>
-      <c r="J79" s="9">
-        <v>46294</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H79" s="10"/>
+      <c r="I79" s="10"/>
+      <c r="J79" s="10"/>
       <c r="K79" s="10" t="s">
         <v>26</v>
       </c>
@@ -6301,59 +6274,55 @@
         <v>26</v>
       </c>
       <c r="M79" s="10" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N79" s="10" t="s">
-        <v>253</v>
+        <v>26</v>
       </c>
       <c r="O79" s="10" t="s">
-        <v>204</v>
+        <v>272</v>
       </c>
       <c r="P79" s="10" t="s">
-        <v>253</v>
-      </c>
-      <c r="Q79" s="9">
-        <v>46294</v>
-      </c>
-      <c r="R79" s="9">
-        <v>46294</v>
-      </c>
-      <c r="S79" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T79" s="10">
-        <v>0</v>
-      </c>
-      <c r="U79" s="11" t="s">
-        <v>60</v>
+        <v>26</v>
+      </c>
+      <c r="Q79" s="10"/>
+      <c r="R79" s="10"/>
+      <c r="S79" s="10"/>
+      <c r="T79" s="10"/>
+      <c r="U79" s="12" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="B80" s="5">
-        <v>46169.66953854167</v>
-      </c>
-      <c r="C80" s="6"/>
+        <v>46169.66960956018</v>
+      </c>
+      <c r="C80" s="5">
+        <v>46209.84488153935</v>
+      </c>
       <c r="D80" s="5">
-        <v>46197.84256122685</v>
+        <v>46209.844928101855</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>206</v>
+        <v>274</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>186</v>
+        <v>235</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="I80" s="6"/>
+        <v>236</v>
+      </c>
+      <c r="I80" s="5">
+        <v>46174</v>
+      </c>
       <c r="J80" s="5">
-        <v>46294</v>
+        <v>46174</v>
       </c>
       <c r="K80" s="6" t="s">
         <v>26</v>
@@ -6365,46 +6334,60 @@
         <v>26</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>275</v>
+        <v>231</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>269</v>
+        <v>133</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="Q80" s="6"/>
-      <c r="R80" s="6"/>
-      <c r="S80" s="6"/>
-      <c r="T80" s="6"/>
-      <c r="U80" s="6"/>
+        <v>241</v>
+      </c>
+      <c r="Q80" s="5">
+        <v>46174</v>
+      </c>
+      <c r="R80" s="5">
+        <v>46174</v>
+      </c>
+      <c r="S80" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="T80" s="6">
+        <v>1</v>
+      </c>
+      <c r="U80" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B81" s="9">
-        <v>46169.669544212964</v>
-      </c>
-      <c r="C81" s="10"/>
+        <v>46169.6696165162</v>
+      </c>
+      <c r="C81" s="9">
+        <v>46209.844589050925</v>
+      </c>
       <c r="D81" s="9">
-        <v>46197.84251650463</v>
+        <v>46209.84471936343</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>211</v>
+        <v>276</v>
       </c>
       <c r="F81" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G81" s="10" t="s">
-        <v>186</v>
+        <v>235</v>
       </c>
       <c r="H81" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="I81" s="10"/>
+        <v>236</v>
+      </c>
+      <c r="I81" s="9">
+        <v>46288</v>
+      </c>
       <c r="J81" s="9">
-        <v>46294</v>
+        <v>46288</v>
       </c>
       <c r="K81" s="10" t="s">
         <v>26</v>
@@ -6416,84 +6399,108 @@
         <v>26</v>
       </c>
       <c r="N81" s="10" t="s">
-        <v>275</v>
+        <v>231</v>
       </c>
       <c r="O81" s="10" t="s">
-        <v>279</v>
+        <v>123</v>
       </c>
       <c r="P81" s="10" t="s">
-        <v>280</v>
-      </c>
-      <c r="Q81" s="10"/>
-      <c r="R81" s="10"/>
-      <c r="S81" s="10"/>
-      <c r="T81" s="10"/>
-      <c r="U81" s="10"/>
+        <v>277</v>
+      </c>
+      <c r="Q81" s="9">
+        <v>46288</v>
+      </c>
+      <c r="R81" s="9">
+        <v>46288</v>
+      </c>
+      <c r="S81" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T81" s="10">
+        <v>1</v>
+      </c>
+      <c r="U81" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="B82" s="5">
-        <v>46169.66960108797</v>
-      </c>
-      <c r="C82" s="6"/>
+        <v>46169.669622939815</v>
+      </c>
+      <c r="C82" s="5">
+        <v>46209.85400761574</v>
+      </c>
       <c r="D82" s="5">
-        <v>46209.85402508102</v>
+        <v>46209.85430440972</v>
       </c>
       <c r="E82" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="F82" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G82" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="H82" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="I82" s="5">
+        <v>46308</v>
+      </c>
+      <c r="J82" s="5">
+        <v>46308</v>
+      </c>
+      <c r="K82" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L82" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M82" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N82" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="F82" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H82" s="6"/>
-      <c r="I82" s="6"/>
-      <c r="J82" s="6"/>
-      <c r="K82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M82" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="N82" s="6" t="s">
-        <v>26</v>
-      </c>
       <c r="O82" s="6" t="s">
-        <v>282</v>
+        <v>142</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q82" s="6"/>
-      <c r="R82" s="6"/>
-      <c r="S82" s="6"/>
-      <c r="T82" s="6"/>
-      <c r="U82" s="12" t="s">
-        <v>66</v>
+        <v>277</v>
+      </c>
+      <c r="Q82" s="5">
+        <v>46308</v>
+      </c>
+      <c r="R82" s="5">
+        <v>46308</v>
+      </c>
+      <c r="S82" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T82" s="6">
+        <v>1</v>
+      </c>
+      <c r="U82" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="B83" s="9">
-        <v>46169.66960956018</v>
-      </c>
-      <c r="C83" s="9">
-        <v>46209.84488153935</v>
-      </c>
+        <v>46169.66962980324</v>
+      </c>
+      <c r="C83" s="10"/>
       <c r="D83" s="9">
-        <v>46209.844928101855</v>
+        <v>46204.86356525463</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="F83" s="10" t="s">
         <v>26</v>
@@ -6505,10 +6512,10 @@
         <v>236</v>
       </c>
       <c r="I83" s="9">
-        <v>46174</v>
+        <v>46287</v>
       </c>
       <c r="J83" s="9">
-        <v>46174</v>
+        <v>46287</v>
       </c>
       <c r="K83" s="10" t="s">
         <v>26</v>
@@ -6523,42 +6530,40 @@
         <v>231</v>
       </c>
       <c r="O83" s="10" t="s">
-        <v>133</v>
+        <v>182</v>
       </c>
       <c r="P83" s="10" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="Q83" s="9">
-        <v>46174</v>
+        <v>46287</v>
       </c>
       <c r="R83" s="9">
-        <v>46174</v>
-      </c>
-      <c r="S83" s="11" t="s">
-        <v>128</v>
+        <v>46287</v>
+      </c>
+      <c r="S83" s="7" t="s">
+        <v>33</v>
       </c>
       <c r="T83" s="10">
-        <v>1</v>
-      </c>
-      <c r="U83" s="7" t="s">
-        <v>27</v>
+        <v>0</v>
+      </c>
+      <c r="U83" s="12" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="B84" s="5">
-        <v>46169.6696165162</v>
-      </c>
-      <c r="C84" s="5">
-        <v>46209.844589050925</v>
-      </c>
+        <v>46169.669635185186</v>
+      </c>
+      <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46209.84471936343</v>
+        <v>46174.84778872685</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>287</v>
+        <v>58</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>26</v>
@@ -6570,10 +6575,10 @@
         <v>236</v>
       </c>
       <c r="I84" s="5">
-        <v>46288</v>
+        <v>46220</v>
       </c>
       <c r="J84" s="5">
-        <v>46288</v>
+        <v>46220</v>
       </c>
       <c r="K84" s="6" t="s">
         <v>26</v>
@@ -6588,58 +6593,50 @@
         <v>231</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>123</v>
+        <v>153</v>
       </c>
       <c r="P84" s="6" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="Q84" s="5">
-        <v>46288</v>
+        <v>46220</v>
       </c>
       <c r="R84" s="5">
-        <v>46288</v>
+        <v>46220</v>
       </c>
       <c r="S84" s="7" t="s">
         <v>33</v>
       </c>
       <c r="T84" s="6">
-        <v>1</v>
-      </c>
-      <c r="U84" s="7" t="s">
-        <v>27</v>
+        <v>0</v>
+      </c>
+      <c r="U84" s="11" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B85" s="9">
-        <v>46169.669622939815</v>
-      </c>
-      <c r="C85" s="9">
-        <v>46209.85400761574</v>
-      </c>
+        <v>46169.66964790509</v>
+      </c>
+      <c r="C85" s="10"/>
       <c r="D85" s="9">
-        <v>46209.85430440972</v>
+        <v>46209.84945282407</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="F85" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G85" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="H85" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="I85" s="9">
-        <v>46308</v>
-      </c>
-      <c r="J85" s="9">
-        <v>46308</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H85" s="10"/>
+      <c r="I85" s="10"/>
+      <c r="J85" s="10"/>
       <c r="K85" s="10" t="s">
         <v>26</v>
       </c>
@@ -6647,61 +6644,51 @@
         <v>26</v>
       </c>
       <c r="M85" s="10" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N85" s="10" t="s">
-        <v>231</v>
+        <v>26</v>
       </c>
       <c r="O85" s="10" t="s">
-        <v>142</v>
+        <v>287</v>
       </c>
       <c r="P85" s="10" t="s">
-        <v>288</v>
-      </c>
-      <c r="Q85" s="9">
-        <v>46308</v>
-      </c>
-      <c r="R85" s="9">
-        <v>46308</v>
-      </c>
-      <c r="S85" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T85" s="10">
-        <v>1</v>
-      </c>
-      <c r="U85" s="7" t="s">
-        <v>27</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q85" s="10"/>
+      <c r="R85" s="10"/>
+      <c r="S85" s="10"/>
+      <c r="T85" s="10"/>
+      <c r="U85" s="10"/>
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="B86" s="5">
-        <v>46169.66962980324</v>
+        <v>46169.66965109954</v>
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="5">
-        <v>46204.86356525463</v>
+        <v>46174.84790094907</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>235</v>
+        <v>91</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>236</v>
+        <v>91</v>
       </c>
       <c r="I86" s="5">
-        <v>46287</v>
+        <v>46294</v>
       </c>
       <c r="J86" s="5">
-        <v>46287</v>
+        <v>46315</v>
       </c>
       <c r="K86" s="6" t="s">
         <v>26</v>
@@ -6713,19 +6700,19 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>231</v>
+        <v>286</v>
       </c>
       <c r="O86" s="6" t="s">
-        <v>182</v>
+        <v>290</v>
       </c>
       <c r="P86" s="6" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="Q86" s="5">
-        <v>46287</v>
+        <v>46294</v>
       </c>
       <c r="R86" s="5">
-        <v>46287</v>
+        <v>46315</v>
       </c>
       <c r="S86" s="7" t="s">
         <v>33</v>
@@ -6733,38 +6720,38 @@
       <c r="T86" s="6">
         <v>0</v>
       </c>
-      <c r="U86" s="12" t="s">
-        <v>66</v>
+      <c r="U86" s="11" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="B87" s="9">
-        <v>46169.669635185186</v>
+        <v>46169.6696568287</v>
       </c>
       <c r="C87" s="10"/>
       <c r="D87" s="9">
-        <v>46174.84778872685</v>
+        <v>46174.84798839121</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>58</v>
+        <v>206</v>
       </c>
       <c r="F87" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G87" s="10" t="s">
-        <v>235</v>
+        <v>91</v>
       </c>
       <c r="H87" s="10" t="s">
-        <v>236</v>
+        <v>91</v>
       </c>
       <c r="I87" s="9">
-        <v>46220</v>
+        <v>46294</v>
       </c>
       <c r="J87" s="9">
-        <v>46220</v>
+        <v>46315</v>
       </c>
       <c r="K87" s="10" t="s">
         <v>26</v>
@@ -6776,53 +6763,51 @@
         <v>26</v>
       </c>
       <c r="N87" s="10" t="s">
-        <v>231</v>
+        <v>289</v>
       </c>
       <c r="O87" s="10" t="s">
-        <v>153</v>
+        <v>292</v>
       </c>
       <c r="P87" s="10" t="s">
-        <v>295</v>
-      </c>
-      <c r="Q87" s="9">
-        <v>46220</v>
-      </c>
-      <c r="R87" s="9">
-        <v>46220</v>
-      </c>
-      <c r="S87" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T87" s="10">
-        <v>0</v>
-      </c>
-      <c r="U87" s="11" t="s">
-        <v>60</v>
-      </c>
+        <v>289</v>
+      </c>
+      <c r="Q87" s="10"/>
+      <c r="R87" s="10"/>
+      <c r="S87" s="10"/>
+      <c r="T87" s="10"/>
+      <c r="U87" s="10"/>
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="B88" s="5">
-        <v>46169.66964790509</v>
-      </c>
-      <c r="C88" s="6"/>
+        <v>46169.669688622685</v>
+      </c>
+      <c r="C88" s="5">
+        <v>46209.84929427083</v>
+      </c>
       <c r="D88" s="5">
-        <v>46209.84945282407</v>
+        <v>46209.8493094213</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="F88" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H88" s="6"/>
-      <c r="I88" s="6"/>
-      <c r="J88" s="6"/>
+        <v>91</v>
+      </c>
+      <c r="H88" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="I88" s="5">
+        <v>46316</v>
+      </c>
+      <c r="J88" s="5">
+        <v>46316</v>
+      </c>
       <c r="K88" s="6" t="s">
         <v>26</v>
       </c>
@@ -6830,36 +6815,46 @@
         <v>26</v>
       </c>
       <c r="M88" s="6" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>26</v>
+        <v>286</v>
       </c>
       <c r="O88" s="6" t="s">
-        <v>298</v>
+        <v>206</v>
       </c>
       <c r="P88" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q88" s="6"/>
-      <c r="R88" s="6"/>
-      <c r="S88" s="6"/>
-      <c r="T88" s="6"/>
-      <c r="U88" s="6"/>
+        <v>286</v>
+      </c>
+      <c r="Q88" s="5">
+        <v>46316</v>
+      </c>
+      <c r="R88" s="5">
+        <v>46316</v>
+      </c>
+      <c r="S88" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T88" s="6">
+        <v>1</v>
+      </c>
+      <c r="U88" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B89" s="9">
-        <v>46169.66965109954</v>
+        <v>46169.66969347223</v>
       </c>
       <c r="C89" s="10"/>
       <c r="D89" s="9">
-        <v>46174.84790094907</v>
+        <v>46209.84459753473</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>300</v>
+        <v>206</v>
       </c>
       <c r="F89" s="10" t="s">
         <v>26</v>
@@ -6870,11 +6865,9 @@
       <c r="H89" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="I89" s="9">
-        <v>46294</v>
-      </c>
+      <c r="I89" s="10"/>
       <c r="J89" s="9">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="K89" s="10" t="s">
         <v>26</v>
@@ -6886,43 +6879,35 @@
         <v>26</v>
       </c>
       <c r="N89" s="10" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="O89" s="10" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="P89" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="Q89" s="9">
-        <v>46294</v>
-      </c>
-      <c r="R89" s="9">
-        <v>46315</v>
-      </c>
-      <c r="S89" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T89" s="10">
-        <v>0</v>
-      </c>
-      <c r="U89" s="11" t="s">
-        <v>60</v>
-      </c>
+      <c r="Q89" s="10"/>
+      <c r="R89" s="10"/>
+      <c r="S89" s="10"/>
+      <c r="T89" s="10"/>
+      <c r="U89" s="10"/>
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="B90" s="5">
-        <v>46169.6696568287</v>
-      </c>
-      <c r="C90" s="6"/>
+        <v>46169.66972681713</v>
+      </c>
+      <c r="C90" s="5">
+        <v>46209.84944726852</v>
+      </c>
       <c r="D90" s="5">
-        <v>46174.84798839121</v>
+        <v>46209.84946481482</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>206</v>
+        <v>299</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>26</v>
@@ -6934,10 +6919,10 @@
         <v>91</v>
       </c>
       <c r="I90" s="5">
-        <v>46294</v>
+        <v>46317</v>
       </c>
       <c r="J90" s="5">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="K90" s="6" t="s">
         <v>26</v>
@@ -6949,35 +6934,43 @@
         <v>26</v>
       </c>
       <c r="N90" s="6" t="s">
-        <v>300</v>
+        <v>286</v>
       </c>
       <c r="O90" s="6" t="s">
-        <v>303</v>
+        <v>206</v>
       </c>
       <c r="P90" s="6" t="s">
-        <v>300</v>
-      </c>
-      <c r="Q90" s="6"/>
-      <c r="R90" s="6"/>
-      <c r="S90" s="6"/>
-      <c r="T90" s="6"/>
-      <c r="U90" s="6"/>
+        <v>286</v>
+      </c>
+      <c r="Q90" s="5">
+        <v>46317</v>
+      </c>
+      <c r="R90" s="5">
+        <v>46317</v>
+      </c>
+      <c r="S90" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T90" s="6">
+        <v>1</v>
+      </c>
+      <c r="U90" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="B91" s="9">
-        <v>46169.669688622685</v>
-      </c>
-      <c r="C91" s="9">
-        <v>46209.84929427083</v>
-      </c>
+        <v>46169.66973180555</v>
+      </c>
+      <c r="C91" s="10"/>
       <c r="D91" s="9">
-        <v>46209.8493094213</v>
+        <v>46209.844891030094</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>305</v>
+        <v>206</v>
       </c>
       <c r="F91" s="10" t="s">
         <v>26</v>
@@ -6989,10 +6982,10 @@
         <v>91</v>
       </c>
       <c r="I91" s="9">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="J91" s="9">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="K91" s="10" t="s">
         <v>26</v>
@@ -7004,43 +6997,33 @@
         <v>26</v>
       </c>
       <c r="N91" s="10" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="O91" s="10" t="s">
-        <v>206</v>
+        <v>301</v>
       </c>
       <c r="P91" s="10" t="s">
-        <v>297</v>
-      </c>
-      <c r="Q91" s="9">
-        <v>46316</v>
-      </c>
-      <c r="R91" s="9">
-        <v>46316</v>
-      </c>
-      <c r="S91" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T91" s="10">
-        <v>1</v>
-      </c>
-      <c r="U91" s="7" t="s">
-        <v>27</v>
-      </c>
+        <v>302</v>
+      </c>
+      <c r="Q91" s="10"/>
+      <c r="R91" s="10"/>
+      <c r="S91" s="10"/>
+      <c r="T91" s="10"/>
+      <c r="U91" s="10"/>
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B92" s="5">
-        <v>46169.66969347223</v>
+        <v>46169.66981054399</v>
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46209.84459753473</v>
+        <v>46174.8478909375</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>206</v>
+        <v>304</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>26</v>
@@ -7051,9 +7034,11 @@
       <c r="H92" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="I92" s="6"/>
+      <c r="I92" s="5">
+        <v>46318</v>
+      </c>
       <c r="J92" s="5">
-        <v>46316</v>
+        <v>46318</v>
       </c>
       <c r="K92" s="6" t="s">
         <v>26</v>
@@ -7065,35 +7050,43 @@
         <v>26</v>
       </c>
       <c r="N92" s="6" t="s">
-        <v>305</v>
+        <v>286</v>
       </c>
       <c r="O92" s="6" t="s">
-        <v>307</v>
+        <v>206</v>
       </c>
       <c r="P92" s="6" t="s">
-        <v>308</v>
-      </c>
-      <c r="Q92" s="6"/>
-      <c r="R92" s="6"/>
-      <c r="S92" s="6"/>
-      <c r="T92" s="6"/>
-      <c r="U92" s="6"/>
+        <v>286</v>
+      </c>
+      <c r="Q92" s="5">
+        <v>46318</v>
+      </c>
+      <c r="R92" s="5">
+        <v>46318</v>
+      </c>
+      <c r="S92" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T92" s="6">
+        <v>0</v>
+      </c>
+      <c r="U92" s="11" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="8" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="B93" s="9">
-        <v>46169.66972681713</v>
-      </c>
-      <c r="C93" s="9">
-        <v>46209.84944726852</v>
-      </c>
+        <v>46169.66981724537</v>
+      </c>
+      <c r="C93" s="10"/>
       <c r="D93" s="9">
-        <v>46209.84946481482</v>
+        <v>46209.85401892361</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>310</v>
+        <v>206</v>
       </c>
       <c r="F93" s="10" t="s">
         <v>26</v>
@@ -7105,10 +7098,10 @@
         <v>91</v>
       </c>
       <c r="I93" s="9">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="J93" s="9">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="K93" s="10" t="s">
         <v>26</v>
@@ -7120,43 +7113,33 @@
         <v>26</v>
       </c>
       <c r="N93" s="10" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="O93" s="10" t="s">
-        <v>206</v>
+        <v>306</v>
       </c>
       <c r="P93" s="10" t="s">
-        <v>297</v>
-      </c>
-      <c r="Q93" s="9">
-        <v>46317</v>
-      </c>
-      <c r="R93" s="9">
-        <v>46317</v>
-      </c>
-      <c r="S93" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T93" s="10">
-        <v>1</v>
-      </c>
-      <c r="U93" s="7" t="s">
-        <v>27</v>
-      </c>
+        <v>307</v>
+      </c>
+      <c r="Q93" s="10"/>
+      <c r="R93" s="10"/>
+      <c r="S93" s="10"/>
+      <c r="T93" s="10"/>
+      <c r="U93" s="10"/>
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="B94" s="5">
-        <v>46169.66973180555</v>
+        <v>46169.669861041664</v>
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46209.844891030094</v>
+        <v>46174.8478862037</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>206</v>
+        <v>309</v>
       </c>
       <c r="F94" s="6" t="s">
         <v>26</v>
@@ -7168,10 +7151,10 @@
         <v>91</v>
       </c>
       <c r="I94" s="5">
-        <v>46317</v>
+        <v>46321</v>
       </c>
       <c r="J94" s="5">
-        <v>46317</v>
+        <v>46321</v>
       </c>
       <c r="K94" s="6" t="s">
         <v>26</v>
@@ -7183,33 +7166,43 @@
         <v>26</v>
       </c>
       <c r="N94" s="6" t="s">
-        <v>310</v>
+        <v>286</v>
       </c>
       <c r="O94" s="6" t="s">
-        <v>312</v>
+        <v>206</v>
       </c>
       <c r="P94" s="6" t="s">
-        <v>313</v>
-      </c>
-      <c r="Q94" s="6"/>
-      <c r="R94" s="6"/>
-      <c r="S94" s="6"/>
-      <c r="T94" s="6"/>
-      <c r="U94" s="6"/>
+        <v>286</v>
+      </c>
+      <c r="Q94" s="5">
+        <v>46321</v>
+      </c>
+      <c r="R94" s="5">
+        <v>46321</v>
+      </c>
+      <c r="S94" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T94" s="6">
+        <v>0</v>
+      </c>
+      <c r="U94" s="11" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="8" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="B95" s="9">
-        <v>46169.66981054399</v>
+        <v>46169.66986724537</v>
       </c>
       <c r="C95" s="10"/>
       <c r="D95" s="9">
-        <v>46174.8478909375</v>
+        <v>46174.84816675926</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>315</v>
+        <v>206</v>
       </c>
       <c r="F95" s="10" t="s">
         <v>26</v>
@@ -7221,10 +7214,10 @@
         <v>91</v>
       </c>
       <c r="I95" s="9">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="J95" s="9">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="K95" s="10" t="s">
         <v>26</v>
@@ -7236,43 +7229,33 @@
         <v>26</v>
       </c>
       <c r="N95" s="10" t="s">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="O95" s="10" t="s">
         <v>206</v>
       </c>
       <c r="P95" s="10" t="s">
-        <v>297</v>
-      </c>
-      <c r="Q95" s="9">
-        <v>46318</v>
-      </c>
-      <c r="R95" s="9">
-        <v>46318</v>
-      </c>
-      <c r="S95" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T95" s="10">
-        <v>0</v>
-      </c>
-      <c r="U95" s="11" t="s">
-        <v>60</v>
-      </c>
+        <v>311</v>
+      </c>
+      <c r="Q95" s="10"/>
+      <c r="R95" s="10"/>
+      <c r="S95" s="10"/>
+      <c r="T95" s="10"/>
+      <c r="U95" s="10"/>
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="B96" s="5">
-        <v>46169.66981724537</v>
+        <v>46169.66990296297</v>
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46209.85401892361</v>
+        <v>46174.84788545139</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>206</v>
+        <v>313</v>
       </c>
       <c r="F96" s="6" t="s">
         <v>26</v>
@@ -7284,10 +7267,10 @@
         <v>91</v>
       </c>
       <c r="I96" s="5">
-        <v>46318</v>
+        <v>46323</v>
       </c>
       <c r="J96" s="5">
-        <v>46318</v>
+        <v>46323</v>
       </c>
       <c r="K96" s="6" t="s">
         <v>26</v>
@@ -7299,33 +7282,43 @@
         <v>26</v>
       </c>
       <c r="N96" s="6" t="s">
-        <v>315</v>
+        <v>286</v>
       </c>
       <c r="O96" s="6" t="s">
-        <v>317</v>
+        <v>206</v>
       </c>
       <c r="P96" s="6" t="s">
-        <v>318</v>
-      </c>
-      <c r="Q96" s="6"/>
-      <c r="R96" s="6"/>
-      <c r="S96" s="6"/>
-      <c r="T96" s="6"/>
-      <c r="U96" s="6"/>
+        <v>314</v>
+      </c>
+      <c r="Q96" s="5">
+        <v>46323</v>
+      </c>
+      <c r="R96" s="5">
+        <v>46323</v>
+      </c>
+      <c r="S96" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T96" s="6">
+        <v>0</v>
+      </c>
+      <c r="U96" s="11" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B97" s="9">
-        <v>46169.669861041664</v>
+        <v>46169.66994555556</v>
       </c>
       <c r="C97" s="10"/>
       <c r="D97" s="9">
-        <v>46174.8478862037</v>
+        <v>46174.848269317125</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>320</v>
+        <v>206</v>
       </c>
       <c r="F97" s="10" t="s">
         <v>26</v>
@@ -7336,11 +7329,9 @@
       <c r="H97" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="I97" s="9">
-        <v>46321</v>
-      </c>
+      <c r="I97" s="10"/>
       <c r="J97" s="9">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="K97" s="10" t="s">
         <v>26</v>
@@ -7352,59 +7343,43 @@
         <v>26</v>
       </c>
       <c r="N97" s="10" t="s">
-        <v>297</v>
+        <v>313</v>
       </c>
       <c r="O97" s="10" t="s">
         <v>206</v>
       </c>
       <c r="P97" s="10" t="s">
-        <v>297</v>
-      </c>
-      <c r="Q97" s="9">
-        <v>46321</v>
-      </c>
-      <c r="R97" s="9">
-        <v>46321</v>
-      </c>
-      <c r="S97" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T97" s="10">
-        <v>0</v>
-      </c>
-      <c r="U97" s="11" t="s">
-        <v>60</v>
-      </c>
+        <v>316</v>
+      </c>
+      <c r="Q97" s="10"/>
+      <c r="R97" s="10"/>
+      <c r="S97" s="10"/>
+      <c r="T97" s="10"/>
+      <c r="U97" s="10"/>
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="B98" s="5">
-        <v>46169.66986724537</v>
+        <v>46169.669978645834</v>
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46174.84816675926</v>
+        <v>46174.82401747685</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>206</v>
+        <v>318</v>
       </c>
       <c r="F98" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G98" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="H98" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="I98" s="5">
-        <v>46321</v>
-      </c>
-      <c r="J98" s="5">
-        <v>46321</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H98" s="6"/>
+      <c r="I98" s="6"/>
+      <c r="J98" s="6"/>
       <c r="K98" s="6" t="s">
         <v>26</v>
       </c>
@@ -7412,16 +7387,16 @@
         <v>26</v>
       </c>
       <c r="M98" s="6" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N98" s="6" t="s">
-        <v>320</v>
+        <v>26</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>206</v>
+        <v>319</v>
       </c>
       <c r="P98" s="6" t="s">
-        <v>322</v>
+        <v>26</v>
       </c>
       <c r="Q98" s="6"/>
       <c r="R98" s="6"/>
@@ -7431,56 +7406,56 @@
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="B99" s="9">
-        <v>46169.66990296297</v>
+        <v>46169.66998244213</v>
       </c>
       <c r="C99" s="10"/>
       <c r="D99" s="9">
-        <v>46174.84788545139</v>
+        <v>46174.84843513889</v>
       </c>
       <c r="E99" s="10" t="s">
+        <v>321</v>
+      </c>
+      <c r="F99" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G99" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="H99" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="I99" s="9">
+        <v>46324</v>
+      </c>
+      <c r="J99" s="9">
+        <v>46324</v>
+      </c>
+      <c r="K99" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="L99" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="M99" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="N99" s="10" t="s">
+        <v>318</v>
+      </c>
+      <c r="O99" s="10" t="s">
         <v>324</v>
       </c>
-      <c r="F99" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G99" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="H99" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="I99" s="9">
-        <v>46323</v>
-      </c>
-      <c r="J99" s="9">
-        <v>46323</v>
-      </c>
-      <c r="K99" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="L99" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="M99" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="N99" s="10" t="s">
-        <v>297</v>
-      </c>
-      <c r="O99" s="10" t="s">
-        <v>206</v>
-      </c>
       <c r="P99" s="10" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="Q99" s="9">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="R99" s="9">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="S99" s="7" t="s">
         <v>33</v>
@@ -7494,14 +7469,14 @@
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B100" s="5">
-        <v>46169.66994555556</v>
+        <v>46169.66998994213</v>
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="5">
-        <v>46174.848269317125</v>
+        <v>46174.84838837963</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>206</v>
@@ -7510,14 +7485,14 @@
         <v>26</v>
       </c>
       <c r="G100" s="6" t="s">
-        <v>91</v>
+        <v>322</v>
       </c>
       <c r="H100" s="6" t="s">
-        <v>91</v>
+        <v>323</v>
       </c>
       <c r="I100" s="6"/>
       <c r="J100" s="5">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="K100" s="6" t="s">
         <v>26</v>
@@ -7529,13 +7504,13 @@
         <v>26</v>
       </c>
       <c r="N100" s="6" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="O100" s="6" t="s">
         <v>206</v>
       </c>
       <c r="P100" s="6" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="Q100" s="6"/>
       <c r="R100" s="6"/>
@@ -7545,27 +7520,31 @@
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B101" s="9">
-        <v>46169.669978645834</v>
+        <v>46170.63118891204</v>
       </c>
       <c r="C101" s="10"/>
       <c r="D101" s="9">
-        <v>46174.82401747685</v>
+        <v>46209.90833168982</v>
       </c>
       <c r="E101" s="10" t="s">
-        <v>329</v>
+        <v>211</v>
       </c>
       <c r="F101" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G101" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="H101" s="10"/>
+        <v>322</v>
+      </c>
+      <c r="H101" s="10" t="s">
+        <v>323</v>
+      </c>
       <c r="I101" s="10"/>
-      <c r="J101" s="10"/>
+      <c r="J101" s="9">
+        <v>46324</v>
+      </c>
       <c r="K101" s="10" t="s">
         <v>26</v>
       </c>
@@ -7573,16 +7552,16 @@
         <v>26</v>
       </c>
       <c r="M101" s="10" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N101" s="10" t="s">
-        <v>26</v>
+        <v>321</v>
       </c>
       <c r="O101" s="10" t="s">
-        <v>330</v>
+        <v>26</v>
       </c>
       <c r="P101" s="10" t="s">
-        <v>26</v>
+        <v>211</v>
       </c>
       <c r="Q101" s="10"/>
       <c r="R101" s="10"/>
@@ -7592,26 +7571,26 @@
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="B102" s="5">
-        <v>46169.66998244213</v>
+        <v>46174.820955891206</v>
       </c>
       <c r="C102" s="6"/>
       <c r="D102" s="5">
-        <v>46174.84843513889</v>
+        <v>46174.848381284726</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>332</v>
+        <v>62</v>
       </c>
       <c r="F102" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G102" s="6" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
       <c r="H102" s="6" t="s">
-        <v>334</v>
+        <v>323</v>
       </c>
       <c r="I102" s="5">
         <v>46324</v>
@@ -7629,56 +7608,46 @@
         <v>26</v>
       </c>
       <c r="N102" s="6" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="O102" s="6" t="s">
-        <v>335</v>
+        <v>62</v>
       </c>
       <c r="P102" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="Q102" s="5">
-        <v>46324</v>
-      </c>
-      <c r="R102" s="5">
-        <v>46324</v>
-      </c>
-      <c r="S102" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T102" s="6">
-        <v>0</v>
-      </c>
-      <c r="U102" s="11" t="s">
-        <v>60</v>
-      </c>
+      <c r="Q102" s="6"/>
+      <c r="R102" s="6"/>
+      <c r="S102" s="6"/>
+      <c r="T102" s="6"/>
+      <c r="U102" s="6"/>
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="B103" s="9">
-        <v>46169.66998994213</v>
+        <v>46169.670044224535</v>
       </c>
       <c r="C103" s="10"/>
       <c r="D103" s="9">
-        <v>46174.84838837963</v>
+        <v>46174.848558831014</v>
       </c>
       <c r="E103" s="10" t="s">
-        <v>206</v>
+        <v>331</v>
       </c>
       <c r="F103" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G103" s="10" t="s">
-        <v>333</v>
+        <v>91</v>
       </c>
       <c r="H103" s="10" t="s">
-        <v>334</v>
+        <v>91</v>
       </c>
       <c r="I103" s="10"/>
       <c r="J103" s="9">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="K103" s="10" t="s">
         <v>26</v>
@@ -7690,46 +7659,56 @@
         <v>26</v>
       </c>
       <c r="N103" s="10" t="s">
-        <v>332</v>
+        <v>318</v>
       </c>
       <c r="O103" s="10" t="s">
         <v>206</v>
       </c>
       <c r="P103" s="10" t="s">
-        <v>337</v>
-      </c>
-      <c r="Q103" s="10"/>
-      <c r="R103" s="10"/>
-      <c r="S103" s="10"/>
-      <c r="T103" s="10"/>
-      <c r="U103" s="10"/>
+        <v>318</v>
+      </c>
+      <c r="Q103" s="9">
+        <v>46325</v>
+      </c>
+      <c r="R103" s="9">
+        <v>46325</v>
+      </c>
+      <c r="S103" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T103" s="10">
+        <v>0</v>
+      </c>
+      <c r="U103" s="11" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="B104" s="5">
-        <v>46170.63118891204</v>
+        <v>46169.670049050925</v>
       </c>
       <c r="C104" s="6"/>
       <c r="D104" s="5">
-        <v>46174.848385474535</v>
+        <v>46174.848527152775</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="F104" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G104" s="6" t="s">
-        <v>333</v>
+        <v>91</v>
       </c>
       <c r="H104" s="6" t="s">
-        <v>334</v>
+        <v>91</v>
       </c>
       <c r="I104" s="6"/>
       <c r="J104" s="5">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="K104" s="6" t="s">
         <v>26</v>
@@ -7741,13 +7720,13 @@
         <v>26</v>
       </c>
       <c r="N104" s="6" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="O104" s="6" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="P104" s="6" t="s">
-        <v>211</v>
+        <v>333</v>
       </c>
       <c r="Q104" s="6"/>
       <c r="R104" s="6"/>
@@ -7757,32 +7736,30 @@
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A105" s="8" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="B105" s="9">
-        <v>46174.820955891206</v>
+        <v>46170.63213679398</v>
       </c>
       <c r="C105" s="10"/>
       <c r="D105" s="9">
-        <v>46174.848381284726</v>
+        <v>46174.848524270834</v>
       </c>
       <c r="E105" s="10" t="s">
-        <v>62</v>
+        <v>211</v>
       </c>
       <c r="F105" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G105" s="10" t="s">
-        <v>333</v>
+        <v>91</v>
       </c>
       <c r="H105" s="10" t="s">
-        <v>334</v>
-      </c>
-      <c r="I105" s="9">
-        <v>46324</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="I105" s="10"/>
       <c r="J105" s="9">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="K105" s="10" t="s">
         <v>26</v>
@@ -7794,13 +7771,13 @@
         <v>26</v>
       </c>
       <c r="N105" s="10" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="O105" s="10" t="s">
-        <v>62</v>
+        <v>211</v>
       </c>
       <c r="P105" s="10" t="s">
-        <v>340</v>
+        <v>211</v>
       </c>
       <c r="Q105" s="10"/>
       <c r="R105" s="10"/>
@@ -7810,17 +7787,17 @@
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="B106" s="5">
-        <v>46169.670044224535</v>
+        <v>46174.82099290509</v>
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46174.848558831014</v>
+        <v>46174.84852028935</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>342</v>
+        <v>329</v>
       </c>
       <c r="F106" s="6" t="s">
         <v>26</v>
@@ -7831,7 +7808,9 @@
       <c r="H106" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="I106" s="6"/>
+      <c r="I106" s="5">
+        <v>46325</v>
+      </c>
       <c r="J106" s="5">
         <v>46325</v>
       </c>
@@ -7845,56 +7824,46 @@
         <v>26</v>
       </c>
       <c r="N106" s="6" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="O106" s="6" t="s">
-        <v>206</v>
+        <v>62</v>
       </c>
       <c r="P106" s="6" t="s">
-        <v>329</v>
-      </c>
-      <c r="Q106" s="5">
-        <v>46325</v>
-      </c>
-      <c r="R106" s="5">
-        <v>46325</v>
-      </c>
-      <c r="S106" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T106" s="6">
-        <v>0</v>
-      </c>
-      <c r="U106" s="11" t="s">
-        <v>60</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="Q106" s="6"/>
+      <c r="R106" s="6"/>
+      <c r="S106" s="6"/>
+      <c r="T106" s="6"/>
+      <c r="U106" s="6"/>
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A107" s="8" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="B107" s="9">
-        <v>46169.670049050925</v>
+        <v>46169.67013976852</v>
       </c>
       <c r="C107" s="10"/>
       <c r="D107" s="9">
-        <v>46174.848527152775</v>
+        <v>46174.84870307871</v>
       </c>
       <c r="E107" s="10" t="s">
-        <v>206</v>
+        <v>337</v>
       </c>
       <c r="F107" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G107" s="10" t="s">
-        <v>91</v>
+        <v>256</v>
       </c>
       <c r="H107" s="10" t="s">
-        <v>91</v>
+        <v>257</v>
       </c>
       <c r="I107" s="10"/>
       <c r="J107" s="9">
-        <v>46325</v>
+        <v>46328</v>
       </c>
       <c r="K107" s="10" t="s">
         <v>26</v>
@@ -7906,46 +7875,58 @@
         <v>26</v>
       </c>
       <c r="N107" s="10" t="s">
-        <v>342</v>
+        <v>318</v>
       </c>
       <c r="O107" s="10" t="s">
         <v>206</v>
       </c>
       <c r="P107" s="10" t="s">
-        <v>344</v>
-      </c>
-      <c r="Q107" s="10"/>
-      <c r="R107" s="10"/>
-      <c r="S107" s="10"/>
-      <c r="T107" s="10"/>
-      <c r="U107" s="10"/>
+        <v>318</v>
+      </c>
+      <c r="Q107" s="9">
+        <v>46328</v>
+      </c>
+      <c r="R107" s="9">
+        <v>46328</v>
+      </c>
+      <c r="S107" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T107" s="10">
+        <v>0</v>
+      </c>
+      <c r="U107" s="11" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
       <c r="B108" s="5">
-        <v>46170.63213679398</v>
+        <v>46169.670151377315</v>
       </c>
       <c r="C108" s="6"/>
       <c r="D108" s="5">
-        <v>46174.848524270834</v>
+        <v>46174.848669872685</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="F108" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G108" s="6" t="s">
-        <v>91</v>
+        <v>256</v>
       </c>
       <c r="H108" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="I108" s="6"/>
+        <v>257</v>
+      </c>
+      <c r="I108" s="5">
+        <v>46328</v>
+      </c>
       <c r="J108" s="5">
-        <v>46325</v>
+        <v>46328</v>
       </c>
       <c r="K108" s="6" t="s">
         <v>26</v>
@@ -7957,13 +7938,13 @@
         <v>26</v>
       </c>
       <c r="N108" s="6" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="O108" s="6" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="P108" s="6" t="s">
-        <v>211</v>
+        <v>339</v>
       </c>
       <c r="Q108" s="6"/>
       <c r="R108" s="6"/>
@@ -7973,32 +7954,32 @@
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A109" s="8" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="B109" s="9">
-        <v>46174.82099290509</v>
+        <v>46170.63285997685</v>
       </c>
       <c r="C109" s="10"/>
       <c r="D109" s="9">
-        <v>46174.84852028935</v>
+        <v>46174.848667314815</v>
       </c>
       <c r="E109" s="10" t="s">
-        <v>340</v>
+        <v>211</v>
       </c>
       <c r="F109" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G109" s="10" t="s">
-        <v>91</v>
+        <v>256</v>
       </c>
       <c r="H109" s="10" t="s">
-        <v>91</v>
+        <v>257</v>
       </c>
       <c r="I109" s="9">
-        <v>46325</v>
+        <v>46328</v>
       </c>
       <c r="J109" s="9">
-        <v>46325</v>
+        <v>46328</v>
       </c>
       <c r="K109" s="10" t="s">
         <v>26</v>
@@ -8010,13 +7991,13 @@
         <v>26</v>
       </c>
       <c r="N109" s="10" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="O109" s="10" t="s">
-        <v>62</v>
+        <v>211</v>
       </c>
       <c r="P109" s="10" t="s">
-        <v>62</v>
+        <v>211</v>
       </c>
       <c r="Q109" s="10"/>
       <c r="R109" s="10"/>
@@ -8026,28 +8007,30 @@
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
-        <v>347</v>
+        <v>341</v>
       </c>
       <c r="B110" s="5">
-        <v>46169.67013976852</v>
+        <v>46174.821024143515</v>
       </c>
       <c r="C110" s="6"/>
       <c r="D110" s="5">
-        <v>46174.84870307871</v>
+        <v>46174.84866336806</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>348</v>
+        <v>62</v>
       </c>
       <c r="F110" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G110" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="H110" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="H110" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="I110" s="6"/>
+      <c r="I110" s="5">
+        <v>46328</v>
+      </c>
       <c r="J110" s="5">
         <v>46328</v>
       </c>
@@ -8061,58 +8044,48 @@
         <v>26</v>
       </c>
       <c r="N110" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="O110" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="O110" s="6" t="s">
-        <v>206</v>
-      </c>
       <c r="P110" s="6" t="s">
-        <v>329</v>
-      </c>
-      <c r="Q110" s="5">
-        <v>46328</v>
-      </c>
-      <c r="R110" s="5">
-        <v>46328</v>
-      </c>
-      <c r="S110" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T110" s="6">
-        <v>0</v>
-      </c>
-      <c r="U110" s="11" t="s">
-        <v>60</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="Q110" s="6"/>
+      <c r="R110" s="6"/>
+      <c r="S110" s="6"/>
+      <c r="T110" s="6"/>
+      <c r="U110" s="6"/>
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A111" s="8" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="B111" s="9">
-        <v>46169.670151377315</v>
+        <v>46169.67021965278</v>
       </c>
       <c r="C111" s="10"/>
       <c r="D111" s="9">
-        <v>46174.848669872685</v>
+        <v>46174.84880980324</v>
       </c>
       <c r="E111" s="10" t="s">
-        <v>206</v>
+        <v>343</v>
       </c>
       <c r="F111" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G111" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="H111" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="H111" s="10" t="s">
-        <v>258</v>
-      </c>
       <c r="I111" s="9">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="J111" s="9">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="K111" s="10" t="s">
         <v>26</v>
@@ -8124,48 +8097,56 @@
         <v>26</v>
       </c>
       <c r="N111" s="10" t="s">
-        <v>348</v>
+        <v>318</v>
       </c>
       <c r="O111" s="10" t="s">
         <v>206</v>
       </c>
       <c r="P111" s="10" t="s">
-        <v>350</v>
-      </c>
-      <c r="Q111" s="10"/>
-      <c r="R111" s="10"/>
-      <c r="S111" s="10"/>
-      <c r="T111" s="10"/>
-      <c r="U111" s="10"/>
+        <v>344</v>
+      </c>
+      <c r="Q111" s="9">
+        <v>46329</v>
+      </c>
+      <c r="R111" s="9">
+        <v>46329</v>
+      </c>
+      <c r="S111" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T111" s="10">
+        <v>0</v>
+      </c>
+      <c r="U111" s="11" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="112" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
-        <v>351</v>
+        <v>345</v>
       </c>
       <c r="B112" s="5">
-        <v>46170.63285997685</v>
+        <v>46169.67022677083</v>
       </c>
       <c r="C112" s="6"/>
       <c r="D112" s="5">
-        <v>46174.848667314815</v>
+        <v>46174.84878571759</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="F112" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G112" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="H112" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="H112" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="I112" s="5">
-        <v>46328</v>
-      </c>
+      <c r="I112" s="6"/>
       <c r="J112" s="5">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="K112" s="6" t="s">
         <v>26</v>
@@ -8177,13 +8158,13 @@
         <v>26</v>
       </c>
       <c r="N112" s="6" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="O112" s="6" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="P112" s="6" t="s">
-        <v>211</v>
+        <v>343</v>
       </c>
       <c r="Q112" s="6"/>
       <c r="R112" s="6"/>
@@ -8193,32 +8174,30 @@
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A113" s="8" t="s">
-        <v>352</v>
+        <v>346</v>
       </c>
       <c r="B113" s="9">
-        <v>46174.821024143515</v>
+        <v>46170.633581828704</v>
       </c>
       <c r="C113" s="10"/>
       <c r="D113" s="9">
-        <v>46174.84866336806</v>
+        <v>46174.84878314815</v>
       </c>
       <c r="E113" s="10" t="s">
-        <v>62</v>
+        <v>211</v>
       </c>
       <c r="F113" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G113" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="H113" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="H113" s="10" t="s">
-        <v>258</v>
-      </c>
-      <c r="I113" s="9">
-        <v>46328</v>
-      </c>
+      <c r="I113" s="10"/>
       <c r="J113" s="9">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="K113" s="10" t="s">
         <v>26</v>
@@ -8230,13 +8209,13 @@
         <v>26</v>
       </c>
       <c r="N113" s="10" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="O113" s="10" t="s">
-        <v>340</v>
+        <v>211</v>
       </c>
       <c r="P113" s="10" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="Q113" s="10"/>
       <c r="R113" s="10"/>
@@ -8246,30 +8225,28 @@
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
-        <v>353</v>
+        <v>347</v>
       </c>
       <c r="B114" s="5">
-        <v>46169.67021965278</v>
+        <v>46174.821057037036</v>
       </c>
       <c r="C114" s="6"/>
       <c r="D114" s="5">
-        <v>46174.84880980324</v>
+        <v>46174.84877914352</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>354</v>
+        <v>62</v>
       </c>
       <c r="F114" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G114" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="H114" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="H114" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="I114" s="5">
-        <v>46329</v>
-      </c>
+      <c r="I114" s="6"/>
       <c r="J114" s="5">
         <v>46329</v>
       </c>
@@ -8283,57 +8260,43 @@
         <v>26</v>
       </c>
       <c r="N114" s="6" t="s">
-        <v>329</v>
+        <v>343</v>
       </c>
       <c r="O114" s="6" t="s">
-        <v>206</v>
+        <v>62</v>
       </c>
       <c r="P114" s="6" t="s">
-        <v>355</v>
-      </c>
-      <c r="Q114" s="5">
-        <v>46329</v>
-      </c>
-      <c r="R114" s="5">
-        <v>46329</v>
-      </c>
-      <c r="S114" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T114" s="6">
-        <v>0</v>
-      </c>
-      <c r="U114" s="11" t="s">
-        <v>60</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q114" s="6"/>
+      <c r="R114" s="6"/>
+      <c r="S114" s="6"/>
+      <c r="T114" s="6"/>
+      <c r="U114" s="6"/>
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A115" s="8" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
       <c r="B115" s="9">
-        <v>46169.67022677083</v>
+        <v>46169.67031616898</v>
       </c>
       <c r="C115" s="10"/>
       <c r="D115" s="9">
-        <v>46174.84878571759</v>
+        <v>46174.82401751158</v>
       </c>
       <c r="E115" s="10" t="s">
-        <v>206</v>
+        <v>349</v>
       </c>
       <c r="F115" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G115" s="10" t="s">
-        <v>257</v>
-      </c>
-      <c r="H115" s="10" t="s">
-        <v>258</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H115" s="10"/>
       <c r="I115" s="10"/>
-      <c r="J115" s="9">
-        <v>46329</v>
-      </c>
+      <c r="J115" s="10"/>
       <c r="K115" s="10" t="s">
         <v>26</v>
       </c>
@@ -8341,16 +8304,16 @@
         <v>26</v>
       </c>
       <c r="M115" s="10" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N115" s="10" t="s">
-        <v>354</v>
+        <v>26</v>
       </c>
       <c r="O115" s="10" t="s">
-        <v>206</v>
+        <v>350</v>
       </c>
       <c r="P115" s="10" t="s">
-        <v>354</v>
+        <v>26</v>
       </c>
       <c r="Q115" s="10"/>
       <c r="R115" s="10"/>
@@ -8360,30 +8323,32 @@
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
       <c r="B116" s="5">
-        <v>46170.633581828704</v>
+        <v>46169.67031976852</v>
       </c>
       <c r="C116" s="6"/>
       <c r="D116" s="5">
-        <v>46174.84878314815</v>
+        <v>46174.84885483797</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>211</v>
+        <v>352</v>
       </c>
       <c r="F116" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G116" s="6" t="s">
-        <v>257</v>
+        <v>353</v>
       </c>
       <c r="H116" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="I116" s="6"/>
+        <v>354</v>
+      </c>
+      <c r="I116" s="5">
+        <v>46330</v>
+      </c>
       <c r="J116" s="5">
-        <v>46329</v>
+        <v>46338</v>
       </c>
       <c r="K116" s="6" t="s">
         <v>26</v>
@@ -8395,46 +8360,58 @@
         <v>26</v>
       </c>
       <c r="N116" s="6" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="O116" s="6" t="s">
-        <v>211</v>
+        <v>343</v>
       </c>
       <c r="P116" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q116" s="6"/>
-      <c r="R116" s="6"/>
-      <c r="S116" s="6"/>
-      <c r="T116" s="6"/>
-      <c r="U116" s="6"/>
+        <v>349</v>
+      </c>
+      <c r="Q116" s="5">
+        <v>46330</v>
+      </c>
+      <c r="R116" s="5">
+        <v>46338</v>
+      </c>
+      <c r="S116" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T116" s="6">
+        <v>0</v>
+      </c>
+      <c r="U116" s="11" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A117" s="8" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="B117" s="9">
-        <v>46174.821057037036</v>
+        <v>46169.6703253125</v>
       </c>
       <c r="C117" s="10"/>
       <c r="D117" s="9">
-        <v>46174.84877914352</v>
+        <v>46192.97339644676</v>
       </c>
       <c r="E117" s="10" t="s">
-        <v>62</v>
+        <v>356</v>
       </c>
       <c r="F117" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G117" s="10" t="s">
-        <v>257</v>
+        <v>69</v>
       </c>
       <c r="H117" s="10" t="s">
-        <v>258</v>
-      </c>
-      <c r="I117" s="10"/>
+        <v>70</v>
+      </c>
+      <c r="I117" s="9">
+        <v>46330</v>
+      </c>
       <c r="J117" s="9">
-        <v>46329</v>
+        <v>46338</v>
       </c>
       <c r="K117" s="10" t="s">
         <v>26</v>
@@ -8446,33 +8423,43 @@
         <v>26</v>
       </c>
       <c r="N117" s="10" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="O117" s="10" t="s">
-        <v>62</v>
+        <v>343</v>
       </c>
       <c r="P117" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q117" s="10"/>
-      <c r="R117" s="10"/>
-      <c r="S117" s="10"/>
-      <c r="T117" s="10"/>
-      <c r="U117" s="10"/>
+        <v>349</v>
+      </c>
+      <c r="Q117" s="9">
+        <v>46330</v>
+      </c>
+      <c r="R117" s="9">
+        <v>46338</v>
+      </c>
+      <c r="S117" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T117" s="10">
+        <v>0</v>
+      </c>
+      <c r="U117" s="11" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="118" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B118" s="5">
-        <v>46169.67031616898</v>
+        <v>46169.670332430556</v>
       </c>
       <c r="C118" s="6"/>
       <c r="D118" s="5">
-        <v>46174.82401751158</v>
+        <v>46174.82401726852</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="F118" s="6" t="s">
         <v>25</v>
@@ -8496,39 +8483,45 @@
         <v>26</v>
       </c>
       <c r="O118" s="6" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="P118" s="6" t="s">
         <v>26</v>
       </c>
       <c r="Q118" s="6"/>
       <c r="R118" s="6"/>
-      <c r="S118" s="6"/>
-      <c r="T118" s="6"/>
-      <c r="U118" s="6"/>
+      <c r="S118" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T118" s="6">
+        <v>0</v>
+      </c>
+      <c r="U118" s="11" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A119" s="8" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B119" s="9">
-        <v>46169.67031976852</v>
+        <v>46169.67033591435</v>
       </c>
       <c r="C119" s="10"/>
       <c r="D119" s="9">
-        <v>46174.84885483797</v>
+        <v>46174.848958703704</v>
       </c>
       <c r="E119" s="10" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="F119" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G119" s="10" t="s">
-        <v>364</v>
+        <v>51</v>
       </c>
       <c r="H119" s="10" t="s">
-        <v>365</v>
+        <v>52</v>
       </c>
       <c r="I119" s="9">
         <v>46330</v>
@@ -8546,13 +8539,13 @@
         <v>26</v>
       </c>
       <c r="N119" s="10" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="O119" s="10" t="s">
-        <v>354</v>
+        <v>343</v>
       </c>
       <c r="P119" s="10" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="Q119" s="9">
         <v>46330</v>
@@ -8572,32 +8565,32 @@
     </row>
     <row r="120" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B120" s="5">
-        <v>46169.6703253125</v>
+        <v>46169.67034748843</v>
       </c>
       <c r="C120" s="6"/>
       <c r="D120" s="5">
-        <v>46192.97339644676</v>
+        <v>46174.84895586806</v>
       </c>
       <c r="E120" s="6" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="F120" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G120" s="6" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="H120" s="6" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="I120" s="5">
-        <v>46330</v>
+        <v>46339</v>
       </c>
       <c r="J120" s="5">
-        <v>46338</v>
+        <v>46349</v>
       </c>
       <c r="K120" s="6" t="s">
         <v>26</v>
@@ -8609,19 +8602,19 @@
         <v>26</v>
       </c>
       <c r="N120" s="6" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="O120" s="6" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="P120" s="6" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="Q120" s="5">
-        <v>46330</v>
+        <v>46339</v>
       </c>
       <c r="R120" s="5">
-        <v>46338</v>
+        <v>46349</v>
       </c>
       <c r="S120" s="7" t="s">
         <v>33</v>
@@ -8630,185 +8623,6 @@
         <v>0</v>
       </c>
       <c r="U120" s="11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="121" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A121" s="8" t="s">
-        <v>368</v>
-      </c>
-      <c r="B121" s="9">
-        <v>46169.670332430556</v>
-      </c>
-      <c r="C121" s="10"/>
-      <c r="D121" s="9">
-        <v>46174.82401726852</v>
-      </c>
-      <c r="E121" s="10" t="s">
-        <v>369</v>
-      </c>
-      <c r="F121" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="G121" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="H121" s="10"/>
-      <c r="I121" s="10"/>
-      <c r="J121" s="10"/>
-      <c r="K121" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="L121" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="M121" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="N121" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="O121" s="10" t="s">
-        <v>370</v>
-      </c>
-      <c r="P121" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q121" s="10"/>
-      <c r="R121" s="10"/>
-      <c r="S121" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T121" s="10">
-        <v>0</v>
-      </c>
-      <c r="U121" s="11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="122" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A122" s="4" t="s">
-        <v>371</v>
-      </c>
-      <c r="B122" s="5">
-        <v>46169.67033591435</v>
-      </c>
-      <c r="C122" s="6"/>
-      <c r="D122" s="5">
-        <v>46174.848958703704</v>
-      </c>
-      <c r="E122" s="6" t="s">
-        <v>372</v>
-      </c>
-      <c r="F122" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G122" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="H122" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="I122" s="5">
-        <v>46330</v>
-      </c>
-      <c r="J122" s="5">
-        <v>46338</v>
-      </c>
-      <c r="K122" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L122" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M122" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N122" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="O122" s="6" t="s">
-        <v>354</v>
-      </c>
-      <c r="P122" s="6" t="s">
-        <v>373</v>
-      </c>
-      <c r="Q122" s="5">
-        <v>46330</v>
-      </c>
-      <c r="R122" s="5">
-        <v>46338</v>
-      </c>
-      <c r="S122" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T122" s="6">
-        <v>0</v>
-      </c>
-      <c r="U122" s="11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="123" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A123" s="8" t="s">
-        <v>374</v>
-      </c>
-      <c r="B123" s="9">
-        <v>46169.67034748843</v>
-      </c>
-      <c r="C123" s="10"/>
-      <c r="D123" s="9">
-        <v>46174.84895586806</v>
-      </c>
-      <c r="E123" s="10" t="s">
-        <v>375</v>
-      </c>
-      <c r="F123" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G123" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="H123" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="I123" s="9">
-        <v>46339</v>
-      </c>
-      <c r="J123" s="9">
-        <v>46349</v>
-      </c>
-      <c r="K123" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="L123" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="M123" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="N123" s="10" t="s">
-        <v>369</v>
-      </c>
-      <c r="O123" s="10" t="s">
-        <v>372</v>
-      </c>
-      <c r="P123" s="10" t="s">
-        <v>369</v>
-      </c>
-      <c r="Q123" s="9">
-        <v>46339</v>
-      </c>
-      <c r="R123" s="9">
-        <v>46349</v>
-      </c>
-      <c r="S123" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="T123" s="10">
-        <v>0</v>
-      </c>
-      <c r="U123" s="11" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-09 19:55 UTC
</commit_message>
<xml_diff>
--- a/data/50001558 - GESVIAL OT4342-4344.xlsx
+++ b/data/50001558 - GESVIAL OT4342-4344.xlsx
@@ -243,9 +243,6 @@
     <t>Ingenieria basica Rodete,Ingenieria Detalle,Ingenieria Basica Motor</t>
   </si>
   <si>
-    <t>Tarea en curso</t>
-  </si>
-  <si>
     <t>1215174266168927</t>
   </si>
   <si>
@@ -391,6 +388,9 @@
   </si>
   <si>
     <t>Materiales corte Laser ot 4342 -4344,Motor ot 4342,rodete ot 4342,Alabe ot 4342</t>
+  </si>
+  <si>
+    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1215174084165958</t>
@@ -2373,9 +2373,11 @@
       <c r="B14" s="5">
         <v>46169.66882583333</v>
       </c>
-      <c r="C14" s="6"/>
+      <c r="C14" s="5">
+        <v>46212.79376377315</v>
+      </c>
       <c r="D14" s="5">
-        <v>46192.97341535879</v>
+        <v>46212.79378054398</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>64</v>
@@ -2410,14 +2412,16 @@
       <c r="Q14" s="6"/>
       <c r="R14" s="6"/>
       <c r="S14" s="6"/>
-      <c r="T14" s="6"/>
-      <c r="U14" s="12" t="s">
-        <v>66</v>
+      <c r="T14" s="6">
+        <v>1</v>
+      </c>
+      <c r="U14" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B15" s="9">
         <v>46169.66899085648</v>
@@ -2429,16 +2433,16 @@
         <v>46192.97339646991</v>
       </c>
       <c r="E15" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="F15" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G15" s="10" t="s">
+      <c r="H15" s="10" t="s">
         <v>69</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>70</v>
       </c>
       <c r="I15" s="9">
         <v>46155</v>
@@ -2450,7 +2454,7 @@
         <v>26</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M15" s="10" t="s">
         <v>26</v>
@@ -2462,7 +2466,7 @@
         <v>40</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Q15" s="9">
         <v>46155</v>
@@ -2482,7 +2486,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B16" s="5">
         <v>46169.66899618055</v>
@@ -2494,16 +2498,16 @@
         <v>46192.97339646991</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G16" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="H16" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="I16" s="5">
         <v>46155</v>
@@ -2515,7 +2519,7 @@
         <v>26</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="M16" s="6" t="s">
         <v>26</v>
@@ -2527,7 +2531,7 @@
         <v>40</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Q16" s="5">
         <v>46155</v>
@@ -2547,7 +2551,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B17" s="9">
         <v>46169.669002106486</v>
@@ -2559,16 +2563,16 @@
         <v>46192.97339675926</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F17" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G17" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="H17" s="10" t="s">
         <v>69</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>70</v>
       </c>
       <c r="I17" s="9">
         <v>46155</v>
@@ -2592,7 +2596,7 @@
         <v>40</v>
       </c>
       <c r="P17" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="Q17" s="9">
         <v>46155</v>
@@ -2612,7 +2616,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B18" s="5">
         <v>46169.66883001158</v>
@@ -2624,7 +2628,7 @@
         <v>46197.64488530092</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>25</v>
@@ -2648,7 +2652,7 @@
         <v>26</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="P18" s="6" t="s">
         <v>26</v>
@@ -2665,7 +2669,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B19" s="9">
         <v>46169.669016053245</v>
@@ -2677,16 +2681,16 @@
         <v>46181.636840625</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F19" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G19" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="H19" s="10" t="s">
         <v>69</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>70</v>
       </c>
       <c r="I19" s="9">
         <v>46157</v>
@@ -2704,13 +2708,13 @@
         <v>26</v>
       </c>
       <c r="N19" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O19" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="P19" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="Q19" s="9">
         <v>46157</v>
@@ -2730,7 +2734,7 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B20" s="5">
         <v>46169.669021423615</v>
@@ -2742,16 +2746,16 @@
         <v>46181.636847222224</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G20" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="H20" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="I20" s="5">
         <v>46167</v>
@@ -2769,13 +2773,13 @@
         <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Q20" s="5">
         <v>46167</v>
@@ -2795,7 +2799,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B21" s="9">
         <v>46169.66902680555</v>
@@ -2807,16 +2811,16 @@
         <v>46181.636854895834</v>
       </c>
       <c r="E21" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G21" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="F21" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G21" s="10" t="s">
-        <v>91</v>
-      </c>
       <c r="H21" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I21" s="9">
         <v>46167</v>
@@ -2834,13 +2838,13 @@
         <v>26</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="Q21" s="9">
         <v>46167</v>
@@ -2860,7 +2864,7 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B22" s="5">
         <v>46169.66903233796</v>
@@ -2872,16 +2876,16 @@
         <v>46206.55341104166</v>
       </c>
       <c r="E22" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="F22" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G22" s="6" t="s">
+      <c r="H22" s="6" t="s">
         <v>95</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>96</v>
       </c>
       <c r="I22" s="5">
         <v>46241</v>
@@ -2899,13 +2903,13 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O22" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="P22" s="6" t="s">
         <v>97</v>
-      </c>
-      <c r="P22" s="6" t="s">
-        <v>98</v>
       </c>
       <c r="Q22" s="5">
         <v>46241</v>
@@ -2925,7 +2929,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B23" s="9">
         <v>46169.669037291664</v>
@@ -2937,16 +2941,16 @@
         <v>46197.644057592595</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F23" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G23" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="H23" s="10" t="s">
         <v>95</v>
-      </c>
-      <c r="H23" s="10" t="s">
-        <v>96</v>
       </c>
       <c r="I23" s="9">
         <v>46241</v>
@@ -2964,13 +2968,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O23" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P23" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q23" s="9">
         <v>46241</v>
@@ -2990,7 +2994,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B24" s="5">
         <v>46169.66904123843</v>
@@ -3002,16 +3006,16 @@
         <v>46197.64420756944</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="H24" s="6" t="s">
         <v>95</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>96</v>
       </c>
       <c r="I24" s="5">
         <v>46241</v>
@@ -3029,13 +3033,13 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="Q24" s="5">
         <v>46241</v>
@@ -3055,7 +3059,7 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B25" s="9">
         <v>46169.66904511574</v>
@@ -3067,16 +3071,16 @@
         <v>46197.64487474537</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="H25" s="10" t="s">
         <v>95</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>96</v>
       </c>
       <c r="I25" s="9">
         <v>46241</v>
@@ -3094,13 +3098,13 @@
         <v>26</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O25" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P25" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="Q25" s="9">
         <v>46241</v>
@@ -3120,7 +3124,7 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B26" s="5">
         <v>46169.66904878472</v>
@@ -3132,16 +3136,16 @@
         <v>46195.60168921296</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="H26" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="I26" s="5">
         <v>46157</v>
@@ -3159,13 +3163,13 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O26" s="6" t="s">
         <v>50</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="Q26" s="5">
         <v>46157</v>
@@ -3185,7 +3189,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B27" s="9">
         <v>46169.66883418981</v>
@@ -3195,7 +3199,7 @@
         <v>46209.82175228009</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>25</v>
@@ -3219,7 +3223,7 @@
         <v>26</v>
       </c>
       <c r="O27" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P27" s="10" t="s">
         <v>26</v>
@@ -3229,7 +3233,7 @@
       <c r="S27" s="10"/>
       <c r="T27" s="10"/>
       <c r="U27" s="12" t="s">
-        <v>66</v>
+        <v>113</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
@@ -3273,13 +3277,13 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="O28" s="6" t="s">
         <v>118</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="Q28" s="5">
         <v>46168</v>
@@ -3341,7 +3345,7 @@
         <v>115</v>
       </c>
       <c r="O29" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="P29" s="10" t="s">
         <v>121</v>
@@ -3460,13 +3464,13 @@
         <v>26</v>
       </c>
       <c r="N31" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="O31" s="10" t="s">
         <v>127</v>
       </c>
       <c r="P31" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="Q31" s="9">
         <v>46168</v>
@@ -3528,7 +3532,7 @@
         <v>126</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P32" s="6" t="s">
         <v>131</v>
@@ -3647,13 +3651,13 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="O34" s="6" t="s">
         <v>137</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="Q34" s="5">
         <v>46161</v>
@@ -3715,7 +3719,7 @@
         <v>136</v>
       </c>
       <c r="O35" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P35" s="10" t="s">
         <v>140</v>
@@ -3893,7 +3897,7 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="O38" s="6" t="s">
         <v>149</v>
@@ -3931,7 +3935,7 @@
         <v>46195.68641299769</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F39" s="10" t="s">
         <v>26</v>
@@ -3961,7 +3965,7 @@
         <v>148</v>
       </c>
       <c r="O39" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="P39" s="10" t="s">
         <v>152</v>
@@ -4014,7 +4018,7 @@
         <v>148</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="P40" s="6" t="s">
         <v>155</v>
@@ -4066,13 +4070,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="O41" s="10" t="s">
         <v>160</v>
       </c>
       <c r="P41" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="Q41" s="9">
         <v>46245</v>
@@ -4134,7 +4138,7 @@
         <v>157</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>163</v>
@@ -4253,7 +4257,7 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="O44" s="6" t="s">
         <v>169</v>
@@ -4291,7 +4295,7 @@
         <v>46199.569896354165</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F45" s="10" t="s">
         <v>26</v>
@@ -4321,7 +4325,7 @@
         <v>168</v>
       </c>
       <c r="O45" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P45" s="10" t="s">
         <v>171</v>
@@ -4376,7 +4380,7 @@
         <v>168</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>174</v>
@@ -4428,7 +4432,7 @@
         <v>26</v>
       </c>
       <c r="N47" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="O47" s="10" t="s">
         <v>179</v>
@@ -4466,7 +4470,7 @@
         <v>46204.863510995376</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
@@ -4496,7 +4500,7 @@
         <v>176</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P48" s="6" t="s">
         <v>181</v>
@@ -4551,7 +4555,7 @@
         <v>176</v>
       </c>
       <c r="O49" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="P49" s="10" t="s">
         <v>184</v>
@@ -4658,7 +4662,7 @@
         <v>26</v>
       </c>
       <c r="N51" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="O51" s="10" t="s">
         <v>191</v>
@@ -4696,7 +4700,7 @@
         <v>46199.57078165509</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>26</v>
@@ -4726,7 +4730,7 @@
         <v>190</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="P52" s="6" t="s">
         <v>193</v>
@@ -4781,7 +4785,7 @@
         <v>190</v>
       </c>
       <c r="O53" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="P53" s="10" t="s">
         <v>196</v>
@@ -4954,7 +4958,7 @@
         <v>201</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="P56" s="6" t="s">
         <v>210</v>
@@ -5009,7 +5013,7 @@
         <v>201</v>
       </c>
       <c r="O57" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="P57" s="10" t="s">
         <v>213</v>
@@ -5209,7 +5213,7 @@
         <v>46209.908330949074</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>26</v>
@@ -5301,13 +5305,13 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>207</v>
       </c>
       <c r="P62" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="Q62" s="6"/>
       <c r="R62" s="6"/>
@@ -6101,7 +6105,7 @@
         <v>0.1</v>
       </c>
       <c r="U75" s="12" t="s">
-        <v>66</v>
+        <v>113</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -6317,7 +6321,7 @@
       <c r="S79" s="10"/>
       <c r="T79" s="10"/>
       <c r="U79" s="12" t="s">
-        <v>66</v>
+        <v>113</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
@@ -6575,7 +6579,7 @@
         <v>0</v>
       </c>
       <c r="U83" s="12" t="s">
-        <v>66</v>
+        <v>113</v>
       </c>
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
@@ -6706,10 +6710,10 @@
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I86" s="5">
         <v>46294</v>
@@ -6769,10 +6773,10 @@
         <v>26</v>
       </c>
       <c r="G87" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H87" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I87" s="9">
         <v>46294</v>
@@ -6824,10 +6828,10 @@
         <v>26</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I88" s="5">
         <v>46316</v>
@@ -6887,10 +6891,10 @@
         <v>26</v>
       </c>
       <c r="G89" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H89" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I89" s="10"/>
       <c r="J89" s="9">
@@ -6940,10 +6944,10 @@
         <v>26</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I90" s="5">
         <v>46317</v>
@@ -7003,10 +7007,10 @@
         <v>26</v>
       </c>
       <c r="G91" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H91" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I91" s="9">
         <v>46317</v>
@@ -7056,10 +7060,10 @@
         <v>26</v>
       </c>
       <c r="G92" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I92" s="5">
         <v>46318</v>
@@ -7119,10 +7123,10 @@
         <v>26</v>
       </c>
       <c r="G93" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H93" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I93" s="9">
         <v>46318</v>
@@ -7172,10 +7176,10 @@
         <v>26</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I94" s="5">
         <v>46321</v>
@@ -7235,10 +7239,10 @@
         <v>26</v>
       </c>
       <c r="G95" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H95" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I95" s="9">
         <v>46321</v>
@@ -7288,10 +7292,10 @@
         <v>26</v>
       </c>
       <c r="G96" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H96" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I96" s="5">
         <v>46323</v>
@@ -7351,10 +7355,10 @@
         <v>26</v>
       </c>
       <c r="G97" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H97" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I97" s="10"/>
       <c r="J97" s="9">
@@ -7667,10 +7671,10 @@
         <v>26</v>
       </c>
       <c r="G103" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H103" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I103" s="10"/>
       <c r="J103" s="9">
@@ -7728,10 +7732,10 @@
         <v>26</v>
       </c>
       <c r="G104" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H104" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I104" s="6"/>
       <c r="J104" s="5">
@@ -7779,10 +7783,10 @@
         <v>26</v>
       </c>
       <c r="G105" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H105" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I105" s="10"/>
       <c r="J105" s="9">
@@ -7830,10 +7834,10 @@
         <v>26</v>
       </c>
       <c r="G106" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H106" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I106" s="5">
         <v>46325</v>
@@ -8429,10 +8433,10 @@
         <v>26</v>
       </c>
       <c r="G117" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="H117" s="10" t="s">
         <v>69</v>
-      </c>
-      <c r="H117" s="10" t="s">
-        <v>70</v>
       </c>
       <c r="I117" s="9">
         <v>46330</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-16 16:39 Chile
</commit_message>
<xml_diff>
--- a/data/50001558 - GESVIAL OT4342-4344.xlsx
+++ b/data/50001558 - GESVIAL OT4342-4344.xlsx
@@ -5343,7 +5343,7 @@
       </c>
       <c r="C63" s="10"/>
       <c r="D63" s="9">
-        <v>46250.34665685185</v>
+        <v>46250.63425142361</v>
       </c>
       <c r="E63" s="10" t="s">
         <v>226</v>
@@ -6671,7 +6671,7 @@
       </c>
       <c r="C85" s="10"/>
       <c r="D85" s="9">
-        <v>46223.56797070602</v>
+        <v>46250.63500270833</v>
       </c>
       <c r="E85" s="10" t="s">
         <v>287</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-09-06 19:15 Chile
</commit_message>
<xml_diff>
--- a/data/50001558 - GESVIAL OT4342-4344.xlsx
+++ b/data/50001558 - GESVIAL OT4342-4344.xlsx
@@ -5953,7 +5953,7 @@
         <v>46209.90925715277</v>
       </c>
       <c r="D73" s="9">
-        <v>46265.171999108796</v>
+        <v>46271.708096064816</v>
       </c>
       <c r="E73" s="10" t="s">
         <v>255</v>
@@ -6071,7 +6071,7 @@
       </c>
       <c r="C75" s="10"/>
       <c r="D75" s="9">
-        <v>46260.587916261575</v>
+        <v>46271.70808619213</v>
       </c>
       <c r="E75" s="10" t="s">
         <v>264</v>
@@ -6187,7 +6187,7 @@
       </c>
       <c r="C77" s="10"/>
       <c r="D77" s="9">
-        <v>46260.587929270834</v>
+        <v>46271.70811479166</v>
       </c>
       <c r="E77" s="10" t="s">
         <v>269</v>

</xml_diff>